<commit_message>
Actualización de reporte RFC
</commit_message>
<xml_diff>
--- a/Metricas/Reportes/RFC_Reporte.xlsx
+++ b/Metricas/Reportes/RFC_Reporte.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alumnosuady-my.sharepoint.com/personal/a23216399_alumnos_uady_mx/Documents/Métricas de SW/proyecto/Plantillas de reportes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_761AB092AD39307846EC1CDA738C62821D196A91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99D9410A-12EC-4545-9217-1C44C11B16D9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35F57FB3-4BE7-4B90-8CC6-C7F5CE1D9C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -34,30 +34,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="63">
   <si>
     <t>Resumen</t>
   </si>
@@ -65,181 +43,187 @@
     <t>Proyecto</t>
   </si>
   <si>
+    <t>Métrica Evaluada</t>
+  </si>
+  <si>
+    <t>RFC</t>
+  </si>
+  <si>
+    <t>Fecha de Medición</t>
+  </si>
+  <si>
+    <t>Herramienta Utilizada</t>
+  </si>
+  <si>
+    <t>CodeMR</t>
+  </si>
+  <si>
+    <t>Responsables</t>
+  </si>
+  <si>
+    <t>Descripción corta de la métrica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de Medición: </t>
+  </si>
+  <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Clase</t>
+  </si>
+  <si>
+    <t>Valor RFC</t>
+  </si>
+  <si>
+    <t>Nivel de Riesgo</t>
+  </si>
+  <si>
+    <t>modelo</t>
+  </si>
+  <si>
+    <t>AccionCasilla.java</t>
+  </si>
+  <si>
+    <t>AccionCasillaTrampa.java</t>
+  </si>
+  <si>
+    <t>AccionCasillaVictoria.java</t>
+  </si>
+  <si>
+    <t>CambioCasillaEventManager.java</t>
+  </si>
+  <si>
+    <t>CambioCasillaListener</t>
+  </si>
+  <si>
+    <t>Dado.java</t>
+  </si>
+  <si>
+    <t>MotorDeTurnos.java</t>
+  </si>
+  <si>
+    <t>MovimientoEventManager.java</t>
+  </si>
+  <si>
+    <t>MovimientoListener</t>
+  </si>
+  <si>
+    <t>Partida.java</t>
+  </si>
+  <si>
+    <t>modelo.cartas</t>
+  </si>
+  <si>
+    <t>Carta.java</t>
+  </si>
+  <si>
+    <t>EfectoConObjetivo.java</t>
+  </si>
+  <si>
+    <t>EfectoSinObjetivo.java</t>
+  </si>
+  <si>
+    <t>Mazo.java</t>
+  </si>
+  <si>
+    <t>TipoCarta.java</t>
+  </si>
+  <si>
+    <t>modelo.cartas.blanco</t>
+  </si>
+  <si>
+    <t>BoogieWoogie.java</t>
+  </si>
+  <si>
+    <t>Plegaria.java</t>
+  </si>
+  <si>
+    <t>modelo.cartas.global</t>
+  </si>
+  <si>
+    <t>DistorsionDelEntorno.java</t>
+  </si>
+  <si>
+    <t>Monzon.java</t>
+  </si>
+  <si>
+    <t>modelo.cartas.maestra</t>
+  </si>
+  <si>
+    <t>CartaTemploDeLirios.java</t>
+  </si>
+  <si>
+    <t>GrilletesDelAlma.java</t>
+  </si>
+  <si>
+    <t>modelo.cartas.propia</t>
+  </si>
+  <si>
+    <t>Flash.java</t>
+  </si>
+  <si>
+    <t>RegresoACasa.java</t>
+  </si>
+  <si>
+    <t>modelo.jugador</t>
+  </si>
+  <si>
+    <t>ColorJugador.java</t>
+  </si>
+  <si>
+    <t>EfectoJugador.java</t>
+  </si>
+  <si>
+    <t>EfectoStun.java</t>
+  </si>
+  <si>
+    <t>EstadoJugador.java</t>
+  </si>
+  <si>
+    <t>Jugador.java</t>
+  </si>
+  <si>
+    <t>modelo.mapa</t>
+  </si>
+  <si>
+    <t>Casilla.java</t>
+  </si>
+  <si>
+    <t>GeneradorDeMapa.java</t>
+  </si>
+  <si>
+    <t>Mapa.java</t>
+  </si>
+  <si>
+    <t>TipoCasilla.java</t>
+  </si>
+  <si>
+    <t>GRAFICAS</t>
+  </si>
+  <si>
+    <t>Gráfica distribución de RFC</t>
+  </si>
+  <si>
+    <t>Gráfica estructura de paquetes RFC</t>
+  </si>
+  <si>
+    <t>Gráfica Sunburst RFC</t>
+  </si>
+  <si>
+    <t>TreeMap RFC</t>
+  </si>
+  <si>
     <t>EBOGE</t>
   </si>
   <si>
-    <t>Métrica Evaluada</t>
-  </si>
-  <si>
-    <t>RFC</t>
-  </si>
-  <si>
-    <t>Fecha de Medición</t>
-  </si>
-  <si>
-    <t>Herramienta Utilizada</t>
-  </si>
-  <si>
-    <t>CodeMR</t>
-  </si>
-  <si>
-    <t>Responsables</t>
-  </si>
-  <si>
-    <t>Descripción corta de la métrica</t>
-  </si>
-  <si>
-    <t>Resumen de lo obtenido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha de Medición: </t>
-  </si>
-  <si>
-    <t>Módulo</t>
-  </si>
-  <si>
-    <t>Clase</t>
-  </si>
-  <si>
-    <t>Valor RFC</t>
-  </si>
-  <si>
-    <t>Nivel de Riesgo</t>
-  </si>
-  <si>
-    <t>modelo</t>
-  </si>
-  <si>
-    <t>AccionCasilla.java</t>
-  </si>
-  <si>
-    <t>AccionCasillaTrampa.java</t>
-  </si>
-  <si>
-    <t>AccionCasillaVictoria.java</t>
-  </si>
-  <si>
-    <t>CambioCasillaEventManager.java</t>
-  </si>
-  <si>
-    <t>CambioCasillaListener</t>
-  </si>
-  <si>
-    <t>Dado.java</t>
-  </si>
-  <si>
-    <t>MotorDeTurnos.java</t>
-  </si>
-  <si>
-    <t>MovimientoEventManager.java</t>
-  </si>
-  <si>
-    <t>MovimientoListener</t>
-  </si>
-  <si>
-    <t>Partida.java</t>
-  </si>
-  <si>
-    <t>modelo.cartas</t>
-  </si>
-  <si>
-    <t>Carta.java</t>
-  </si>
-  <si>
-    <t>EfectoConObjetivo.java</t>
-  </si>
-  <si>
-    <t>EfectoSinObjetivo.java</t>
-  </si>
-  <si>
-    <t>Mazo.java</t>
-  </si>
-  <si>
-    <t>TipoCarta.java</t>
-  </si>
-  <si>
-    <t>modelo.cartas.blanco</t>
-  </si>
-  <si>
-    <t>BoogieWoogie.java</t>
-  </si>
-  <si>
-    <t>Plegaria.java</t>
-  </si>
-  <si>
-    <t>modelo.cartas.global</t>
-  </si>
-  <si>
-    <t>DistorsionDelEntorno.java</t>
-  </si>
-  <si>
-    <t>Monzon.java</t>
-  </si>
-  <si>
-    <t>modelo.cartas.maestra</t>
-  </si>
-  <si>
-    <t>CartaTemploDeLirios.java</t>
-  </si>
-  <si>
-    <t>GrilletesDelAlma.java</t>
-  </si>
-  <si>
-    <t>modelo.cartas.propia</t>
-  </si>
-  <si>
-    <t>Flash.java</t>
-  </si>
-  <si>
-    <t>RegresoACasa.java</t>
-  </si>
-  <si>
-    <t>modelo.jugador</t>
-  </si>
-  <si>
-    <t>ColorJugador.java</t>
-  </si>
-  <si>
-    <t>EfectoJugador.java</t>
-  </si>
-  <si>
-    <t>EfectoStun.java</t>
-  </si>
-  <si>
-    <t>EstadoJugador.java</t>
-  </si>
-  <si>
-    <t>Jugador.java</t>
-  </si>
-  <si>
-    <t>modelo.mapa</t>
-  </si>
-  <si>
-    <t>Casilla.java</t>
-  </si>
-  <si>
-    <t>GeneradorDeMapa.java</t>
-  </si>
-  <si>
-    <t>Mapa.java</t>
-  </si>
-  <si>
-    <t>TipoCasilla.java</t>
-  </si>
-  <si>
-    <t>GRAFICAS</t>
-  </si>
-  <si>
-    <t>Gráfica distribución de RFC</t>
-  </si>
-  <si>
-    <t>Gráfica estructura de paquetes RFC</t>
-  </si>
-  <si>
-    <t>Gráfica Sunburst RFC</t>
-  </si>
-  <si>
-    <t>TreeMap RFC</t>
+    <t>Erick Ricardo Vega Nolasco</t>
+  </si>
+  <si>
+    <t>Se analizó un total de 32 clases pertenecientes a los módulos centrales del sistema EBOGE. Los resultados indican que la arquitectura mantiene un nivel de acoplamiento y complejidad de comunicación muy bajo, 31 clases (96.8%), en el nivel de riesgo Muy bajo. En el nivel de riesgo Bajo-medio se identifico 1 clase (3.125%): MotorDeTurnos.java, siendo esta la que presenta el valor más alto del sistema con un RFC de 72. Dado que ninguna clase alcanzó los niveles de riesgo Medio, Alto o Muy alto, el diseño no presenta fragilidad por exceso de dependencias o sobrecarga de responsabilidades, lo que facilita su prueba y mantenimiento continuo.</t>
+  </si>
+  <si>
+    <t>La métrica RFC (Response For a Class) mide el conjunto de métodos que pueden ser ejecutados en respuesta a un mensaje recibido por un objeto de la clase, incluyendo tanto sus propios métodos como aquellos llamados externamente desde otras clases.</t>
   </si>
 </sst>
 </file>
@@ -262,10 +246,6 @@
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <b/>
       <sz val="26"/>
       <color rgb="FFFFFFFF"/>
@@ -280,12 +260,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0D2137"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7A9ABF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -320,6 +294,16 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="18">
@@ -426,25 +410,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF1B4F72"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF1B4F72"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -457,19 +428,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF1B4F72"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAAC4D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAAC4D9"/>
       </bottom>
       <diagonal/>
     </border>
@@ -502,19 +460,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF1B4F72"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAAC4D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF1B4F72"/>
@@ -524,19 +469,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFAAC4D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF1B4F72"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF1B4F72"/>
       </bottom>
       <diagonal/>
     </border>
@@ -565,19 +497,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF1B4F72"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAAC4D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color rgb="FF1B4F72"/>
@@ -588,17 +507,6 @@
       <bottom style="thin">
         <color rgb="FFAAC4D9"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF1B4F72"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAAC4D9"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -659,119 +567,244 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1B4F72"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAC4D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAC4D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1B4F72"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAC4D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1B4F72"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAC4D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAC4D9"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B4F72"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1B4F72"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B4F72"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFAAC4D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="11" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -903,173 +936,183 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>-1</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3132665</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>43786</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90B3A038-98C9-FF50-7BEF-2E24FB3F3EFD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2489199" y="1151467"/>
+          <a:ext cx="7789333" cy="8104052"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="228600" cy="228600"/>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3454400</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>1793</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image4.png">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBAF14E2-48DA-FBA3-7E1E-36DD2A235AFB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12208933" y="1151467"/>
+          <a:ext cx="8111067" cy="8062059"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="209550" cy="228600"/>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3561169</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image3.png">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E745947-7C57-7EE7-F460-384B4C85A121}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2489200" y="9736667"/>
+          <a:ext cx="8217836" cy="8060266"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>135466</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="361950" cy="228600"/>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>4642890</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>207197</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="image1.png">
+        <xdr:cNvPr id="5" name="Imagen 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C796701-2E0E-B9CD-E0FE-C9CE74C9EFF7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12208933" y="10820399"/>
+          <a:ext cx="9299557" cy="4813065"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1281,88 +1324,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="5:6" ht="14.4">
-      <c r="E1" s="25"/>
-      <c r="F1" s="26"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="28"/>
     </row>
     <row r="2" spans="5:6" ht="33.6">
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="28"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="5:6" ht="14.4">
-      <c r="E3" s="25"/>
-      <c r="F3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="5" spans="5:6" ht="14.4">
       <c r="E5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="5:6" ht="14.4">
       <c r="E6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="7" spans="5:6" ht="14.4">
       <c r="E7" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="3">
-        <v>46277</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="8" spans="5:6" ht="14.4">
       <c r="E8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="9" spans="5:6" ht="14.4">
       <c r="E9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="F9" s="54" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="11" spans="5:6" ht="15.6">
       <c r="E11" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="26"/>
+        <v>8</v>
+      </c>
+      <c r="F11" s="28"/>
     </row>
     <row r="12" spans="5:6" ht="86.25" customHeight="1">
-      <c r="E12" s="30"/>
-      <c r="F12" s="26"/>
-    </row>
+      <c r="E12" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="53"/>
+    </row>
+    <row r="13" spans="5:6" ht="14.4"/>
     <row r="14" spans="5:6" ht="15.6">
-      <c r="E14" s="31" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" s="32"/>
-    </row>
-    <row r="15" spans="5:6" ht="78" customHeight="1">
-      <c r="E15" s="33"/>
-      <c r="F15" s="26"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31"/>
+    </row>
+    <row r="15" spans="5:6" ht="162.6" customHeight="1">
+      <c r="E15" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1379,504 +1427,504 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="6">
-        <v>46277</v>
+      <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="5">
+        <v>46168</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="3" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="7" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="str">
+      <c r="D4" s="7" t="str">
         <f t="shared" ref="D4:D35" si="0">IF(C4&gt;=200,"Muy alto",IF(C4&gt;=150,"Alto",IF(C4&gt;=100,"Medio",IF(C4&gt;=50,"Bajo","Muy bajo"))))</f>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>7</v>
       </c>
-      <c r="D5" s="8" t="str">
+      <c r="D5" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="8">
+      <c r="A6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="7">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="str">
+      <c r="D6" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="8">
+      <c r="A7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="7">
         <v>6</v>
       </c>
-      <c r="D7" s="8" t="str">
+      <c r="D7" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8">
+      <c r="A8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="7">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="str">
+      <c r="D8" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A9" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="8">
+      <c r="A9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="7">
         <v>4</v>
       </c>
-      <c r="D9" s="8" t="str">
+      <c r="D9" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="8">
+      <c r="A10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="7">
         <v>72</v>
       </c>
-      <c r="D10" s="8" t="str">
-        <f t="shared" si="0"/>
+      <c r="D10" s="7" t="str">
+        <f>IF(C10&gt;=200,"Muy alto",IF(C10&gt;=150,"Alto",IF(C10&gt;=100,"Medio",IF(C10&gt;=50,"Bajo","Muy bajo"))))</f>
         <v>Bajo</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A11" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="8">
+      <c r="A11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="7">
         <v>6</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="D11" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A12" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="8">
+      <c r="A12" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="7">
         <v>1</v>
       </c>
-      <c r="D12" s="8" t="str">
+      <c r="D12" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="8">
+      <c r="A13" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="7">
         <v>31</v>
       </c>
-      <c r="D13" s="8" t="str">
+      <c r="D13" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="10">
+      <c r="A14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="9">
         <v>4</v>
       </c>
-      <c r="D14" s="8" t="str">
+      <c r="D14" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>1</v>
       </c>
-      <c r="D15" s="8" t="str">
+      <c r="D15" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A16" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="10">
+      <c r="A16" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="9">
         <v>1</v>
       </c>
-      <c r="D16" s="8" t="str">
+      <c r="D16" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A17" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="10">
+      <c r="A17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="9">
         <v>14</v>
       </c>
-      <c r="D17" s="8" t="str">
+      <c r="D17" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A18" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="10">
+      <c r="A18" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="9">
         <v>0</v>
       </c>
-      <c r="D18" s="8" t="str">
+      <c r="D18" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A19" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="12">
+      <c r="A19" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="11">
         <v>12</v>
       </c>
-      <c r="D19" s="8" t="str">
+      <c r="D19" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="12">
+      <c r="C20" s="11">
         <v>13</v>
       </c>
-      <c r="D20" s="8" t="str">
+      <c r="D20" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A21" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="14">
+      <c r="A21" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="13">
         <v>23</v>
       </c>
-      <c r="D21" s="8" t="str">
+      <c r="D21" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <v>14</v>
       </c>
-      <c r="D22" s="8" t="str">
+      <c r="D22" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A23" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="16">
+      <c r="A23" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="15">
         <v>17</v>
       </c>
-      <c r="D23" s="8" t="str">
+      <c r="D23" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="16">
+      <c r="C24" s="15">
         <v>24</v>
       </c>
-      <c r="D24" s="8" t="str">
+      <c r="D24" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A25" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="18">
+      <c r="A25" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" s="17">
         <v>15</v>
       </c>
-      <c r="D25" s="8" t="str">
+      <c r="D25" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="18">
+      <c r="C26" s="17">
         <v>16</v>
       </c>
-      <c r="D26" s="8" t="str">
+      <c r="D26" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A27" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="20">
+      <c r="A27" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="19">
         <v>3</v>
       </c>
-      <c r="D27" s="8" t="str">
+      <c r="D27" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="20">
+      <c r="C28" s="19">
         <v>5</v>
       </c>
-      <c r="D28" s="8" t="str">
+      <c r="D28" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A29" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="C29" s="20">
+      <c r="A29" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="19">
         <v>13</v>
       </c>
-      <c r="D29" s="8" t="str">
+      <c r="D29" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A30" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C30" s="20">
+      <c r="A30" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="19">
         <v>0</v>
       </c>
-      <c r="D30" s="8" t="str">
+      <c r="D30" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A31" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" s="20">
+      <c r="A31" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="19">
         <v>41</v>
       </c>
-      <c r="D31" s="8" t="str">
+      <c r="D31" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A32" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="22">
+      <c r="A32" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" s="21">
         <v>5</v>
       </c>
-      <c r="D32" s="8" t="str">
+      <c r="D32" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C33" s="22">
+      <c r="C33" s="21">
         <v>13</v>
       </c>
-      <c r="D33" s="8" t="str">
+      <c r="D33" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A34" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="C34" s="22">
+      <c r="A34" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" s="21">
         <v>14</v>
       </c>
-      <c r="D34" s="8" t="str">
+      <c r="D34" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A35" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C35" s="22">
+      <c r="A35" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" s="21">
         <v>6</v>
       </c>
-      <c r="D35" s="8" t="str">
+      <c r="D35" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Muy bajo</v>
       </c>
@@ -2898,450 +2946,448 @@
   <sheetData>
     <row r="1" spans="4:8" ht="13.5" customHeight="1"/>
     <row r="2" spans="4:8" ht="49.5" customHeight="1">
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="40"/>
+    </row>
+    <row r="3" spans="4:8" ht="27.75" customHeight="1">
+      <c r="D3" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="50"/>
+      <c r="G3" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="44"/>
-    </row>
-    <row r="3" spans="4:8" ht="27.75" customHeight="1">
-      <c r="D3" s="34" t="s">
+      <c r="H3" s="50"/>
+    </row>
+    <row r="4" spans="4:8" ht="18" customHeight="1" thickBot="1">
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="33"/>
+    </row>
+    <row r="5" spans="4:8" ht="18" customHeight="1">
+      <c r="D5" s="43"/>
+      <c r="E5" s="44"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
+    </row>
+    <row r="6" spans="4:8" ht="18" customHeight="1">
+      <c r="D6" s="43"/>
+      <c r="E6" s="44"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="35"/>
+    </row>
+    <row r="7" spans="4:8" ht="18" customHeight="1">
+      <c r="D7" s="43"/>
+      <c r="E7" s="44"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
+    </row>
+    <row r="8" spans="4:8" ht="18" customHeight="1">
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
+    </row>
+    <row r="9" spans="4:8" ht="18" customHeight="1">
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="35"/>
+    </row>
+    <row r="10" spans="4:8" ht="18" customHeight="1">
+      <c r="D10" s="43"/>
+      <c r="E10" s="44"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="35"/>
+    </row>
+    <row r="11" spans="4:8" ht="18" customHeight="1">
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="35"/>
+    </row>
+    <row r="12" spans="4:8" ht="18" customHeight="1">
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="35"/>
+    </row>
+    <row r="13" spans="4:8" ht="18" customHeight="1">
+      <c r="D13" s="43"/>
+      <c r="E13" s="44"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35"/>
+    </row>
+    <row r="14" spans="4:8" ht="18" customHeight="1">
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="35"/>
+    </row>
+    <row r="15" spans="4:8" ht="18" customHeight="1">
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="35"/>
+    </row>
+    <row r="16" spans="4:8" ht="18" customHeight="1">
+      <c r="D16" s="43"/>
+      <c r="E16" s="44"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="35"/>
+    </row>
+    <row r="17" spans="4:8" ht="18" customHeight="1">
+      <c r="D17" s="43"/>
+      <c r="E17" s="44"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
+    </row>
+    <row r="18" spans="4:8" ht="18" customHeight="1">
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="35"/>
+    </row>
+    <row r="19" spans="4:8" ht="18" customHeight="1">
+      <c r="D19" s="43"/>
+      <c r="E19" s="44"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="35"/>
+    </row>
+    <row r="20" spans="4:8" ht="18" customHeight="1">
+      <c r="D20" s="43"/>
+      <c r="E20" s="44"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="35"/>
+    </row>
+    <row r="21" spans="4:8" ht="18" customHeight="1">
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="35"/>
+    </row>
+    <row r="22" spans="4:8" ht="18" customHeight="1">
+      <c r="D22" s="43"/>
+      <c r="E22" s="44"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="35"/>
+    </row>
+    <row r="23" spans="4:8" ht="18" customHeight="1">
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="35"/>
+    </row>
+    <row r="24" spans="4:8" ht="18" customHeight="1">
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="35"/>
+    </row>
+    <row r="25" spans="4:8" ht="18" customHeight="1">
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="35"/>
+    </row>
+    <row r="26" spans="4:8" ht="18" customHeight="1">
+      <c r="D26" s="43"/>
+      <c r="E26" s="44"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="35"/>
+    </row>
+    <row r="27" spans="4:8" ht="18" customHeight="1">
+      <c r="D27" s="43"/>
+      <c r="E27" s="44"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="35"/>
+    </row>
+    <row r="28" spans="4:8" ht="18" customHeight="1">
+      <c r="D28" s="43"/>
+      <c r="E28" s="44"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="35"/>
+    </row>
+    <row r="29" spans="4:8" ht="18" customHeight="1">
+      <c r="D29" s="43"/>
+      <c r="E29" s="44"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="35"/>
+    </row>
+    <row r="30" spans="4:8" ht="18" customHeight="1">
+      <c r="D30" s="43"/>
+      <c r="E30" s="44"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="35"/>
+    </row>
+    <row r="31" spans="4:8" ht="18" customHeight="1">
+      <c r="D31" s="43"/>
+      <c r="E31" s="44"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="35"/>
+    </row>
+    <row r="32" spans="4:8" ht="18" customHeight="1">
+      <c r="D32" s="43"/>
+      <c r="E32" s="44"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="35"/>
+    </row>
+    <row r="33" spans="4:8" ht="18" customHeight="1">
+      <c r="D33" s="43"/>
+      <c r="E33" s="44"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="35"/>
+    </row>
+    <row r="34" spans="4:8" ht="18" customHeight="1">
+      <c r="D34" s="43"/>
+      <c r="E34" s="44"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="35"/>
+    </row>
+    <row r="35" spans="4:8" ht="18" customHeight="1">
+      <c r="D35" s="43"/>
+      <c r="E35" s="44"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="35"/>
+    </row>
+    <row r="36" spans="4:8" ht="18" customHeight="1">
+      <c r="D36" s="43"/>
+      <c r="E36" s="44"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="35"/>
+    </row>
+    <row r="37" spans="4:8" ht="18" customHeight="1" thickBot="1">
+      <c r="D37" s="45"/>
+      <c r="E37" s="46"/>
+      <c r="G37" s="36"/>
+      <c r="H37" s="37"/>
+    </row>
+    <row r="38" spans="4:8" ht="13.5" customHeight="1" thickBot="1">
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+    </row>
+    <row r="39" spans="4:8" ht="27.75" customHeight="1">
+      <c r="D39" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="35"/>
-      <c r="G3" s="34" t="s">
+      <c r="E39" s="50"/>
+      <c r="G39" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="35"/>
-    </row>
-    <row r="4" spans="4:8" ht="18" customHeight="1">
-      <c r="D4" s="45" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="E4" s="37"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="37"/>
-    </row>
-    <row r="5" spans="4:8" ht="18" customHeight="1">
-      <c r="D5" s="38"/>
-      <c r="E5" s="39"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-    </row>
-    <row r="6" spans="4:8" ht="18" customHeight="1">
-      <c r="D6" s="38"/>
-      <c r="E6" s="39"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="39"/>
-    </row>
-    <row r="7" spans="4:8" ht="18" customHeight="1">
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="39"/>
-    </row>
-    <row r="8" spans="4:8" ht="18" customHeight="1">
-      <c r="D8" s="38"/>
-      <c r="E8" s="39"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="39"/>
-    </row>
-    <row r="9" spans="4:8" ht="18" customHeight="1">
-      <c r="D9" s="38"/>
-      <c r="E9" s="39"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="39"/>
-    </row>
-    <row r="10" spans="4:8" ht="18" customHeight="1">
-      <c r="D10" s="38"/>
-      <c r="E10" s="39"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="39"/>
-    </row>
-    <row r="11" spans="4:8" ht="18" customHeight="1">
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
-      <c r="G11" s="38"/>
-      <c r="H11" s="39"/>
-    </row>
-    <row r="12" spans="4:8" ht="18" customHeight="1">
-      <c r="D12" s="38"/>
-      <c r="E12" s="39"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="39"/>
-    </row>
-    <row r="13" spans="4:8" ht="18" customHeight="1">
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="39"/>
-    </row>
-    <row r="14" spans="4:8" ht="18" customHeight="1">
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="39"/>
-    </row>
-    <row r="15" spans="4:8" ht="18" customHeight="1">
-      <c r="D15" s="38"/>
-      <c r="E15" s="39"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="39"/>
-    </row>
-    <row r="16" spans="4:8" ht="18" customHeight="1">
-      <c r="D16" s="38"/>
-      <c r="E16" s="39"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="39"/>
-    </row>
-    <row r="17" spans="4:8" ht="18" customHeight="1">
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="39"/>
-    </row>
-    <row r="18" spans="4:8" ht="18" customHeight="1">
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="39"/>
-    </row>
-    <row r="19" spans="4:8" ht="18" customHeight="1">
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
-    </row>
-    <row r="20" spans="4:8" ht="18" customHeight="1">
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="39"/>
-    </row>
-    <row r="21" spans="4:8" ht="18" customHeight="1">
-      <c r="D21" s="38"/>
-      <c r="E21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="39"/>
-    </row>
-    <row r="22" spans="4:8" ht="18" customHeight="1">
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="39"/>
-    </row>
-    <row r="23" spans="4:8" ht="18" customHeight="1">
-      <c r="D23" s="38"/>
-      <c r="E23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="39"/>
-    </row>
-    <row r="24" spans="4:8" ht="18" customHeight="1">
-      <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="39"/>
-    </row>
-    <row r="25" spans="4:8" ht="18" customHeight="1">
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="39"/>
-    </row>
-    <row r="26" spans="4:8" ht="18" customHeight="1">
-      <c r="D26" s="38"/>
-      <c r="E26" s="39"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="39"/>
-    </row>
-    <row r="27" spans="4:8" ht="18" customHeight="1">
-      <c r="D27" s="38"/>
-      <c r="E27" s="39"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
-    </row>
-    <row r="28" spans="4:8" ht="18" customHeight="1">
-      <c r="D28" s="38"/>
-      <c r="E28" s="39"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="39"/>
-    </row>
-    <row r="29" spans="4:8" ht="18" customHeight="1">
-      <c r="D29" s="38"/>
-      <c r="E29" s="39"/>
-      <c r="G29" s="38"/>
-      <c r="H29" s="39"/>
-    </row>
-    <row r="30" spans="4:8" ht="18" customHeight="1">
-      <c r="D30" s="38"/>
-      <c r="E30" s="39"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="39"/>
-    </row>
-    <row r="31" spans="4:8" ht="18" customHeight="1">
-      <c r="D31" s="38"/>
-      <c r="E31" s="39"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="39"/>
-    </row>
-    <row r="32" spans="4:8" ht="18" customHeight="1">
-      <c r="D32" s="38"/>
-      <c r="E32" s="39"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="39"/>
-    </row>
-    <row r="33" spans="4:8" ht="18" customHeight="1">
-      <c r="D33" s="38"/>
-      <c r="E33" s="39"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="39"/>
-    </row>
-    <row r="34" spans="4:8" ht="18" customHeight="1">
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="39"/>
-    </row>
-    <row r="35" spans="4:8" ht="18" customHeight="1">
-      <c r="D35" s="38"/>
-      <c r="E35" s="39"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="39"/>
-    </row>
-    <row r="36" spans="4:8" ht="18" customHeight="1">
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="39"/>
-    </row>
-    <row r="37" spans="4:8" ht="18" customHeight="1">
-      <c r="D37" s="40"/>
-      <c r="E37" s="41"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="41"/>
-    </row>
-    <row r="38" spans="4:8" ht="13.5" customHeight="1">
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-    </row>
-    <row r="39" spans="4:8" ht="27.75" customHeight="1">
-      <c r="D39" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="E39" s="35"/>
-      <c r="G39" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="H39" s="35"/>
+      <c r="H39" s="50"/>
     </row>
     <row r="40" spans="4:8" ht="18" customHeight="1">
-      <c r="D40" s="46"/>
-      <c r="E40" s="37"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="37"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="33"/>
+      <c r="G40" s="48"/>
+      <c r="H40" s="33"/>
     </row>
     <row r="41" spans="4:8" ht="18" customHeight="1">
-      <c r="D41" s="38"/>
-      <c r="E41" s="39"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="39"/>
+      <c r="D41" s="34"/>
+      <c r="E41" s="35"/>
+      <c r="G41" s="34"/>
+      <c r="H41" s="35"/>
     </row>
     <row r="42" spans="4:8" ht="18" customHeight="1">
-      <c r="D42" s="38"/>
-      <c r="E42" s="39"/>
-      <c r="G42" s="38"/>
-      <c r="H42" s="39"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="35"/>
+      <c r="G42" s="34"/>
+      <c r="H42" s="35"/>
     </row>
     <row r="43" spans="4:8" ht="18" customHeight="1">
-      <c r="D43" s="38"/>
-      <c r="E43" s="39"/>
-      <c r="G43" s="38"/>
-      <c r="H43" s="39"/>
+      <c r="D43" s="34"/>
+      <c r="E43" s="35"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="35"/>
     </row>
     <row r="44" spans="4:8" ht="18" customHeight="1">
-      <c r="D44" s="38"/>
-      <c r="E44" s="39"/>
-      <c r="G44" s="38"/>
-      <c r="H44" s="39"/>
+      <c r="D44" s="34"/>
+      <c r="E44" s="35"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="35"/>
     </row>
     <row r="45" spans="4:8" ht="18" customHeight="1">
-      <c r="D45" s="38"/>
-      <c r="E45" s="39"/>
-      <c r="G45" s="38"/>
-      <c r="H45" s="39"/>
+      <c r="D45" s="34"/>
+      <c r="E45" s="35"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="35"/>
     </row>
     <row r="46" spans="4:8" ht="18" customHeight="1">
-      <c r="D46" s="38"/>
-      <c r="E46" s="39"/>
-      <c r="G46" s="38"/>
-      <c r="H46" s="39"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="35"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="35"/>
     </row>
     <row r="47" spans="4:8" ht="18" customHeight="1">
-      <c r="D47" s="38"/>
-      <c r="E47" s="39"/>
-      <c r="G47" s="38"/>
-      <c r="H47" s="39"/>
+      <c r="D47" s="34"/>
+      <c r="E47" s="35"/>
+      <c r="G47" s="34"/>
+      <c r="H47" s="35"/>
     </row>
     <row r="48" spans="4:8" ht="18" customHeight="1">
-      <c r="D48" s="38"/>
-      <c r="E48" s="39"/>
-      <c r="G48" s="38"/>
-      <c r="H48" s="39"/>
+      <c r="D48" s="34"/>
+      <c r="E48" s="35"/>
+      <c r="G48" s="34"/>
+      <c r="H48" s="35"/>
     </row>
     <row r="49" spans="4:8" ht="18" customHeight="1">
-      <c r="D49" s="38"/>
-      <c r="E49" s="39"/>
-      <c r="G49" s="38"/>
-      <c r="H49" s="39"/>
+      <c r="D49" s="34"/>
+      <c r="E49" s="35"/>
+      <c r="G49" s="34"/>
+      <c r="H49" s="35"/>
     </row>
     <row r="50" spans="4:8" ht="18" customHeight="1">
-      <c r="D50" s="38"/>
-      <c r="E50" s="39"/>
-      <c r="G50" s="38"/>
-      <c r="H50" s="39"/>
+      <c r="D50" s="34"/>
+      <c r="E50" s="35"/>
+      <c r="G50" s="34"/>
+      <c r="H50" s="35"/>
     </row>
     <row r="51" spans="4:8" ht="18" customHeight="1">
-      <c r="D51" s="38"/>
-      <c r="E51" s="39"/>
-      <c r="G51" s="38"/>
-      <c r="H51" s="39"/>
+      <c r="D51" s="34"/>
+      <c r="E51" s="35"/>
+      <c r="G51" s="34"/>
+      <c r="H51" s="35"/>
     </row>
     <row r="52" spans="4:8" ht="18" customHeight="1">
-      <c r="D52" s="38"/>
-      <c r="E52" s="39"/>
-      <c r="G52" s="38"/>
-      <c r="H52" s="39"/>
+      <c r="D52" s="34"/>
+      <c r="E52" s="35"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="35"/>
     </row>
     <row r="53" spans="4:8" ht="18" customHeight="1">
-      <c r="D53" s="38"/>
-      <c r="E53" s="39"/>
-      <c r="G53" s="38"/>
-      <c r="H53" s="39"/>
+      <c r="D53" s="34"/>
+      <c r="E53" s="35"/>
+      <c r="G53" s="34"/>
+      <c r="H53" s="35"/>
     </row>
     <row r="54" spans="4:8" ht="18" customHeight="1">
-      <c r="D54" s="38"/>
-      <c r="E54" s="39"/>
-      <c r="G54" s="38"/>
-      <c r="H54" s="39"/>
+      <c r="D54" s="34"/>
+      <c r="E54" s="35"/>
+      <c r="G54" s="34"/>
+      <c r="H54" s="35"/>
     </row>
     <row r="55" spans="4:8" ht="18" customHeight="1">
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
-      <c r="G55" s="38"/>
-      <c r="H55" s="39"/>
+      <c r="D55" s="34"/>
+      <c r="E55" s="35"/>
+      <c r="G55" s="34"/>
+      <c r="H55" s="35"/>
     </row>
     <row r="56" spans="4:8" ht="18" customHeight="1">
-      <c r="D56" s="38"/>
-      <c r="E56" s="39"/>
-      <c r="G56" s="38"/>
-      <c r="H56" s="39"/>
+      <c r="D56" s="34"/>
+      <c r="E56" s="35"/>
+      <c r="G56" s="34"/>
+      <c r="H56" s="35"/>
     </row>
     <row r="57" spans="4:8" ht="18" customHeight="1">
-      <c r="D57" s="38"/>
-      <c r="E57" s="39"/>
-      <c r="G57" s="38"/>
-      <c r="H57" s="39"/>
+      <c r="D57" s="34"/>
+      <c r="E57" s="35"/>
+      <c r="G57" s="34"/>
+      <c r="H57" s="35"/>
     </row>
     <row r="58" spans="4:8" ht="18" customHeight="1">
-      <c r="D58" s="38"/>
-      <c r="E58" s="39"/>
-      <c r="G58" s="38"/>
-      <c r="H58" s="39"/>
+      <c r="D58" s="34"/>
+      <c r="E58" s="35"/>
+      <c r="G58" s="34"/>
+      <c r="H58" s="35"/>
     </row>
     <row r="59" spans="4:8" ht="18" customHeight="1">
-      <c r="D59" s="38"/>
-      <c r="E59" s="39"/>
-      <c r="G59" s="38"/>
-      <c r="H59" s="39"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="35"/>
+      <c r="G59" s="34"/>
+      <c r="H59" s="35"/>
     </row>
     <row r="60" spans="4:8" ht="18" customHeight="1">
-      <c r="D60" s="38"/>
-      <c r="E60" s="39"/>
-      <c r="G60" s="38"/>
-      <c r="H60" s="39"/>
+      <c r="D60" s="34"/>
+      <c r="E60" s="35"/>
+      <c r="G60" s="34"/>
+      <c r="H60" s="35"/>
     </row>
     <row r="61" spans="4:8" ht="18" customHeight="1">
-      <c r="D61" s="38"/>
-      <c r="E61" s="39"/>
-      <c r="G61" s="38"/>
-      <c r="H61" s="39"/>
+      <c r="D61" s="34"/>
+      <c r="E61" s="35"/>
+      <c r="G61" s="34"/>
+      <c r="H61" s="35"/>
     </row>
     <row r="62" spans="4:8" ht="18" customHeight="1">
-      <c r="D62" s="38"/>
-      <c r="E62" s="39"/>
-      <c r="G62" s="38"/>
-      <c r="H62" s="39"/>
+      <c r="D62" s="34"/>
+      <c r="E62" s="35"/>
+      <c r="G62" s="34"/>
+      <c r="H62" s="35"/>
     </row>
     <row r="63" spans="4:8" ht="18" customHeight="1">
-      <c r="D63" s="38"/>
-      <c r="E63" s="39"/>
-      <c r="G63" s="38"/>
-      <c r="H63" s="39"/>
+      <c r="D63" s="34"/>
+      <c r="E63" s="35"/>
+      <c r="G63" s="34"/>
+      <c r="H63" s="35"/>
     </row>
     <row r="64" spans="4:8" ht="18" customHeight="1">
-      <c r="D64" s="38"/>
-      <c r="E64" s="39"/>
-      <c r="G64" s="38"/>
-      <c r="H64" s="39"/>
+      <c r="D64" s="34"/>
+      <c r="E64" s="35"/>
+      <c r="G64" s="34"/>
+      <c r="H64" s="35"/>
     </row>
     <row r="65" spans="4:8" ht="18" customHeight="1">
-      <c r="D65" s="38"/>
-      <c r="E65" s="39"/>
-      <c r="G65" s="38"/>
-      <c r="H65" s="39"/>
+      <c r="D65" s="34"/>
+      <c r="E65" s="35"/>
+      <c r="G65" s="34"/>
+      <c r="H65" s="35"/>
     </row>
     <row r="66" spans="4:8" ht="18" customHeight="1">
-      <c r="D66" s="38"/>
-      <c r="E66" s="39"/>
-      <c r="G66" s="38"/>
-      <c r="H66" s="39"/>
+      <c r="D66" s="34"/>
+      <c r="E66" s="35"/>
+      <c r="G66" s="34"/>
+      <c r="H66" s="35"/>
     </row>
     <row r="67" spans="4:8" ht="18" customHeight="1">
-      <c r="D67" s="38"/>
-      <c r="E67" s="39"/>
-      <c r="G67" s="38"/>
-      <c r="H67" s="39"/>
+      <c r="D67" s="34"/>
+      <c r="E67" s="35"/>
+      <c r="G67" s="34"/>
+      <c r="H67" s="35"/>
     </row>
     <row r="68" spans="4:8" ht="18" customHeight="1">
-      <c r="D68" s="38"/>
-      <c r="E68" s="39"/>
-      <c r="G68" s="38"/>
-      <c r="H68" s="39"/>
+      <c r="D68" s="34"/>
+      <c r="E68" s="35"/>
+      <c r="G68" s="34"/>
+      <c r="H68" s="35"/>
     </row>
     <row r="69" spans="4:8" ht="18" customHeight="1">
-      <c r="D69" s="38"/>
-      <c r="E69" s="39"/>
-      <c r="G69" s="38"/>
-      <c r="H69" s="39"/>
+      <c r="D69" s="34"/>
+      <c r="E69" s="35"/>
+      <c r="G69" s="34"/>
+      <c r="H69" s="35"/>
     </row>
     <row r="70" spans="4:8" ht="18" customHeight="1">
-      <c r="D70" s="38"/>
-      <c r="E70" s="39"/>
-      <c r="G70" s="38"/>
-      <c r="H70" s="39"/>
+      <c r="D70" s="34"/>
+      <c r="E70" s="35"/>
+      <c r="G70" s="34"/>
+      <c r="H70" s="35"/>
     </row>
     <row r="71" spans="4:8" ht="18" customHeight="1">
-      <c r="D71" s="38"/>
-      <c r="E71" s="39"/>
-      <c r="G71" s="38"/>
-      <c r="H71" s="39"/>
+      <c r="D71" s="34"/>
+      <c r="E71" s="35"/>
+      <c r="G71" s="34"/>
+      <c r="H71" s="35"/>
     </row>
     <row r="72" spans="4:8" ht="18" customHeight="1">
-      <c r="D72" s="38"/>
-      <c r="E72" s="39"/>
-      <c r="G72" s="38"/>
-      <c r="H72" s="39"/>
+      <c r="D72" s="34"/>
+      <c r="E72" s="35"/>
+      <c r="G72" s="34"/>
+      <c r="H72" s="35"/>
     </row>
     <row r="73" spans="4:8" ht="18" customHeight="1">
-      <c r="D73" s="40"/>
-      <c r="E73" s="41"/>
-      <c r="G73" s="40"/>
-      <c r="H73" s="41"/>
+      <c r="D73" s="36"/>
+      <c r="E73" s="37"/>
+      <c r="G73" s="36"/>
+      <c r="H73" s="37"/>
     </row>
     <row r="74" spans="4:8" ht="13.5" customHeight="1"/>
     <row r="75" spans="4:8" ht="14.25" customHeight="1"/>
@@ -4272,15 +4318,15 @@
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="G4:H37"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:E37"/>
+    <mergeCell ref="D40:E73"/>
     <mergeCell ref="G40:H73"/>
-    <mergeCell ref="D2:H2"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G3:H3"/>
-    <mergeCell ref="D4:E37"/>
-    <mergeCell ref="G4:H37"/>
+    <mergeCell ref="G39:H39"/>
     <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E73"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>